<commit_message>
created schematics, and logic driagram
</commit_message>
<xml_diff>
--- a/doc/2.Document Annexe/JDT_2510_RegulationChauffage_Mendes.xlsx
+++ b/doc/2.Document Annexe/JDT_2510_RegulationChauffage_Mendes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduvaud-my.sharepoint.com/personal/py13jta_eduvaud_ch/Documents/00_Diplome/2510_RegulationChauffage/doc/2.Document Annexe/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="186" documentId="8_{4277F192-9065-4C14-9BEA-4A138BE84FE7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{09653C62-4CA3-4213-9539-CB60268A1635}"/>
+  <xr:revisionPtr revIDLastSave="191" documentId="8_{4277F192-9065-4C14-9BEA-4A138BE84FE7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{25F40E88-8733-4112-BEE4-EDF2C692EE88}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -871,7 +871,7 @@
       <c r="C5" s="28"/>
       <c r="D5" s="11">
         <f>SUM(C12:I12)</f>
-        <v>0.27083333333333326</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="E5" s="12">
         <f>SUM(C21:I21)</f>
@@ -895,7 +895,7 @@
       </c>
       <c r="J5" s="12">
         <f>SUM(D5:I5)</f>
-        <v>0.27083333333333326</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="K5" s="3"/>
     </row>
@@ -978,7 +978,9 @@
       <c r="C9" s="18">
         <v>0.41666666666666669</v>
       </c>
-      <c r="D9" s="18"/>
+      <c r="D9" s="18">
+        <v>0.33333333333333331</v>
+      </c>
       <c r="E9" s="18"/>
       <c r="F9" s="18"/>
       <c r="G9" s="18"/>
@@ -992,7 +994,9 @@
       <c r="C10" s="18">
         <v>0.72916666666666663</v>
       </c>
-      <c r="D10" s="18"/>
+      <c r="D10" s="18">
+        <v>0.70833333333333337</v>
+      </c>
       <c r="E10" s="18"/>
       <c r="F10" s="18"/>
       <c r="G10" s="18"/>
@@ -1006,7 +1010,9 @@
       <c r="C11" s="19">
         <v>4.1666666666666664E-2</v>
       </c>
-      <c r="D11" s="19"/>
+      <c r="D11" s="19">
+        <v>4.1666666666666664E-2</v>
+      </c>
       <c r="E11" s="19"/>
       <c r="F11" s="19"/>
       <c r="G11" s="19"/>
@@ -1023,11 +1029,11 @@
         <v>0.27083333333333326</v>
       </c>
       <c r="D12" s="21">
-        <f t="shared" ref="D12:I12" si="1">D10-D9-D11</f>
-        <v>0</v>
+        <f>D10-D9-D11</f>
+        <v>0.33333333333333337</v>
       </c>
       <c r="E12" s="21">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="D12:I12" si="1">E10-E9-E11</f>
         <v>0</v>
       </c>
       <c r="F12" s="21">

</xml_diff>

<commit_message>
finsihed schmatic version 2.0
</commit_message>
<xml_diff>
--- a/doc/2.Document Annexe/JDT_2510_RegulationChauffage_Mendes.xlsx
+++ b/doc/2.Document Annexe/JDT_2510_RegulationChauffage_Mendes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduvaud-my.sharepoint.com/personal/py13jta_eduvaud_ch/Documents/00_Diplome/2510_RegulationChauffage/doc/2.Document Annexe/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="226" documentId="8_{4277F192-9065-4C14-9BEA-4A138BE84FE7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{B588768A-73F5-4FDB-88AF-C5EA37E321C2}"/>
+  <xr:revisionPtr revIDLastSave="256" documentId="8_{4277F192-9065-4C14-9BEA-4A138BE84FE7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{C22D6F8A-7258-4AC7-8174-6C50F0ACAEE4}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="29">
   <si>
     <t>NOTES</t>
   </si>
@@ -116,6 +116,45 @@
 Recherche sur l'entrée et la schématique liées.
 Recherche sur l'etage ADC et choix du composants et la technologie
 Documentation </t>
+  </si>
+  <si>
+    <t>Fin recherche composant ADC
+Dimensionnement ADC
+Dimensionnement et ajout des I/O du CM5
+Ajout de l'USB
+Meeting de design avec retour sur les différents éléments</t>
+  </si>
+  <si>
+    <t>ADC prix ok
+Ajout USB pour programmation 
+Ethernet en 2 paires 
+Passage du relais sur carte fille</t>
+  </si>
+  <si>
+    <t>Design carte fille
+Ajout des relais
+Recherche solution pour le mux
+Ajout des réseau de résistance
+Début rapport
+Création PV 22.08.2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solution MUX complex, influence de la résitance interne sur le réseau. </t>
+  </si>
+  <si>
+    <t>Solution pour le mux proposée
+Reflection etage de sortie 24V
+Liens des schémas
+Rapport 
+PV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mux cher 15.- ? Meillieur solution ?
+Sortie 24V doivent lire une tension ou injecter un courant ? Influence sur le systèmes actif ? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revue de schéma
+</t>
   </si>
 </sst>
 </file>
@@ -126,7 +165,7 @@
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="166" formatCode="[$-40C]dddd"/>
-    <numFmt numFmtId="168" formatCode="[hh]:mm"/>
+    <numFmt numFmtId="167" formatCode="[hh]:mm"/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
@@ -372,6 +411,12 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -386,12 +431,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -474,8 +513,8 @@
       <xdr:rowOff>132291</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>196011</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>2533965</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>541923</xdr:rowOff>
     </xdr:to>
@@ -789,20 +828,22 @@
     <col min="4" max="4" width="37.875" customWidth="1"/>
     <col min="5" max="5" width="45" customWidth="1"/>
     <col min="6" max="6" width="44.5" customWidth="1"/>
-    <col min="7" max="9" width="30.625" customWidth="1"/>
+    <col min="7" max="7" width="47" customWidth="1"/>
+    <col min="8" max="8" width="46.875" customWidth="1"/>
+    <col min="9" max="9" width="47.875" customWidth="1"/>
     <col min="10" max="10" width="29" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
@@ -865,20 +906,20 @@
       <c r="AF2" s="1"/>
     </row>
     <row r="3" spans="1:32" s="5" customFormat="1" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
     </row>
     <row r="4" spans="1:32" s="3" customFormat="1" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="26"/>
+      <c r="C4" s="28"/>
       <c r="D4" s="12" t="s">
         <v>15</v>
       </c>
@@ -902,37 +943,37 @@
       </c>
     </row>
     <row r="5" spans="1:32" s="4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="27">
+      <c r="B5" s="29">
         <v>45887</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="29">
+      <c r="C5" s="29"/>
+      <c r="D5" s="24">
         <f>SUM(C12:I12)</f>
-        <v>1.802083333333333</v>
-      </c>
-      <c r="E5" s="30">
+        <v>2.177083333333333</v>
+      </c>
+      <c r="E5" s="25">
         <f>SUM(C21:I21)</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="30">
+        <v>1.1041666666666667</v>
+      </c>
+      <c r="F5" s="25">
         <f>SUM(D30:I30)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="30">
+      <c r="G5" s="25">
         <f>SUM(D39:I39)</f>
         <v>0</v>
       </c>
-      <c r="H5" s="30">
+      <c r="H5" s="25">
         <f>SUM(D48:I48)</f>
         <v>0</v>
       </c>
-      <c r="I5" s="30">
+      <c r="I5" s="25">
         <f>SUM(D57:I57)</f>
         <v>0</v>
       </c>
-      <c r="J5" s="30">
+      <c r="J5" s="25">
         <f>SUM(D5:I5)</f>
-        <v>1.802083333333333</v>
+        <v>3.28125</v>
       </c>
       <c r="K5" s="3"/>
     </row>
@@ -945,7 +986,7 @@
       <c r="G6" s="9"/>
     </row>
     <row r="7" spans="1:32" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="24">
+      <c r="B7" s="26">
         <v>1</v>
       </c>
       <c r="C7" s="13">
@@ -978,7 +1019,7 @@
       </c>
     </row>
     <row r="8" spans="1:32" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="24"/>
+      <c r="B8" s="26"/>
       <c r="C8" s="14">
         <f>B5</f>
         <v>45887</v>
@@ -1028,7 +1069,9 @@
         <v>0.34375</v>
       </c>
       <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
+      <c r="I9" s="16">
+        <v>0.45833333333333331</v>
+      </c>
     </row>
     <row r="10" spans="1:32" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="15" t="s">
@@ -1050,7 +1093,9 @@
         <v>0.8125</v>
       </c>
       <c r="H10" s="16"/>
-      <c r="I10" s="16"/>
+      <c r="I10" s="16">
+        <v>0.91666666666666663</v>
+      </c>
     </row>
     <row r="11" spans="1:32" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="15" t="s">
@@ -1072,7 +1117,9 @@
         <v>4.1666666666666664E-2</v>
       </c>
       <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
+      <c r="I11" s="17">
+        <v>8.3333333333333329E-2</v>
+      </c>
       <c r="J11" s="11"/>
     </row>
     <row r="12" spans="1:32" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1105,7 +1152,7 @@
       </c>
       <c r="I12" s="19">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="13" spans="1:32" ht="212.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1121,10 +1168,16 @@
       <c r="E13" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
+      <c r="F13" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="G13" s="21" t="s">
+        <v>24</v>
+      </c>
       <c r="H13" s="21"/>
-      <c r="I13" s="21"/>
+      <c r="I13" s="21" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="14" spans="1:32" ht="76.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="15" t="s">
@@ -1139,10 +1192,16 @@
       <c r="E14" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
+      <c r="F14" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="G14" s="21" t="s">
+        <v>25</v>
+      </c>
       <c r="H14" s="21"/>
-      <c r="I14" s="21"/>
+      <c r="I14" s="21" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="15" spans="1:32" ht="21" x14ac:dyDescent="0.35">
       <c r="B15" s="22"/>
@@ -1155,7 +1214,7 @@
       <c r="I15" s="23"/>
     </row>
     <row r="16" spans="1:32" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="24">
+      <c r="B16" s="26">
         <v>2</v>
       </c>
       <c r="C16" s="13">
@@ -1188,7 +1247,7 @@
       </c>
     </row>
     <row r="17" spans="2:10" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="24"/>
+      <c r="B17" s="26"/>
       <c r="C17" s="14">
         <f>I8+1</f>
         <v>45894</v>
@@ -1222,9 +1281,15 @@
       <c r="B18" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
+      <c r="C18" s="16">
+        <v>0.34375</v>
+      </c>
+      <c r="D18" s="16">
+        <v>0.34375</v>
+      </c>
+      <c r="E18" s="16">
+        <v>0.34375</v>
+      </c>
       <c r="F18" s="16"/>
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
@@ -1234,9 +1299,15 @@
       <c r="B19" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
+      <c r="C19" s="16">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="D19" s="16">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="E19" s="16">
+        <v>0.71875</v>
+      </c>
       <c r="F19" s="16"/>
       <c r="G19" s="16"/>
       <c r="H19" s="16"/>
@@ -1246,9 +1317,15 @@
       <c r="B20" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
+      <c r="C20" s="17">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="D20" s="17">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="E20" s="17">
+        <v>4.1666666666666664E-2</v>
+      </c>
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
       <c r="H20" s="17"/>
@@ -1261,15 +1338,15 @@
       </c>
       <c r="C21" s="19">
         <f>C19-C18-C20</f>
-        <v>0</v>
+        <v>0.38541666666666669</v>
       </c>
       <c r="D21" s="19">
         <f>D19-D18-D20</f>
-        <v>0</v>
+        <v>0.38541666666666669</v>
       </c>
       <c r="E21" s="19">
         <f t="shared" ref="E21:I21" si="3">E19-E18-E20</f>
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="F21" s="19">
         <f t="shared" si="3"/>
@@ -1292,7 +1369,9 @@
       <c r="B22" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="C22" s="21"/>
+      <c r="C22" s="21" t="s">
+        <v>28</v>
+      </c>
       <c r="D22" s="21"/>
       <c r="E22" s="21"/>
       <c r="F22" s="21"/>
@@ -1323,7 +1402,7 @@
       <c r="I24" s="22"/>
     </row>
     <row r="25" spans="2:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="24">
+      <c r="B25" s="26">
         <v>3</v>
       </c>
       <c r="C25" s="13">
@@ -1356,7 +1435,7 @@
       </c>
     </row>
     <row r="26" spans="2:10" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="B26" s="24"/>
+      <c r="B26" s="26"/>
       <c r="C26" s="14">
         <f>I17+1</f>
         <v>45901</v>
@@ -1490,7 +1569,7 @@
       <c r="I33" s="22"/>
     </row>
     <row r="34" spans="2:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="24">
+      <c r="B34" s="26">
         <v>4</v>
       </c>
       <c r="C34" s="13">
@@ -1523,7 +1602,7 @@
       </c>
     </row>
     <row r="35" spans="2:9" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="B35" s="24"/>
+      <c r="B35" s="26"/>
       <c r="C35" s="14">
         <f>I26+1</f>
         <v>45908</v>
@@ -1657,7 +1736,7 @@
       <c r="I42" s="22"/>
     </row>
     <row r="43" spans="2:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="24">
+      <c r="B43" s="26">
         <v>5</v>
       </c>
       <c r="C43" s="13">
@@ -1690,7 +1769,7 @@
       </c>
     </row>
     <row r="44" spans="2:9" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="B44" s="24"/>
+      <c r="B44" s="26"/>
       <c r="C44" s="14">
         <f>I35+1</f>
         <v>45915</v>
@@ -1824,7 +1903,7 @@
       <c r="I51" s="22"/>
     </row>
     <row r="52" spans="2:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="24">
+      <c r="B52" s="26">
         <v>6</v>
       </c>
       <c r="C52" s="13">
@@ -1857,7 +1936,7 @@
       </c>
     </row>
     <row r="53" spans="2:9" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="B53" s="24"/>
+      <c r="B53" s="26"/>
       <c r="C53" s="14">
         <f>I44+1</f>
         <v>45922</v>

</xml_diff>